<commit_message>
Re-render all books with split spin archetypes + Greenblatt Magic Formula
Regenerated the 18 render-managed workbooks (and NMS candidates csv) so the
new arch_spinoff_value / arch_spinoff_quality / arch_greenblatt_magic
archetypes surface in the per-archetype, country, segment, and top-N books.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Pk8K7QpC1m36MYjRwkTznS
</commit_message>
<xml_diff>
--- a/nms_multibagger_candidates_midcap_plus.xlsx
+++ b/nms_multibagger_candidates_midcap_plus.xlsx
@@ -658,7 +658,7 @@
     <row r="9" ht="22" customHeight="1">
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>This shortlist filters the 4,154 multibagger candidates in the NMS sub-universe (mcap &lt; ~$2B, RED-verdicted names excluded). Each name is assigned a conviction tier based on its archetype-count, inflection-cluster density and asymmetry score. STRICT (210) = 5+ archetypes firing AND 3+ inflection signals AND asymmetry &gt;= 0.40. STRONG (198) = 3+ archetypes AND 3+ inflection signals AND asymmetry &gt;= 0.35. CANDIDATE (3746) = the broader funnel - 3+ archetypes or 4+ inflection signals at asymmetry &gt;= 0.35. (Multi-archetype gates are calibrated to the current 69-archetype taxonomy.) Within each tier, names are ranked by confirmed entry-today asymmetry (asymmetry_score x qual_multiplier x post-rally factor x confirmation multiplier (1 + 0.20 x confirm_overall + 0.10 x buyback_score)).</t>
+          <t>This shortlist filters the 4,155 multibagger candidates in the NMS sub-universe (mcap &lt; ~$2B, RED-verdicted names excluded). Each name is assigned a conviction tier based on its archetype-count, inflection-cluster density and asymmetry score. STRICT (210) = 5+ archetypes firing AND 3+ inflection signals AND asymmetry &gt;= 0.40. STRONG (198) = 3+ archetypes AND 3+ inflection signals AND asymmetry &gt;= 0.35. CANDIDATE (3747) = the broader funnel - 3+ archetypes or 4+ inflection signals at asymmetry &gt;= 0.35. (Multi-archetype gates are calibrated to the current 69-archetype taxonomy.) Within each tier, names are ranked by confirmed entry-today asymmetry (asymmetry_score x qual_multiplier x post-rally factor x confirmation multiplier (1 + 0.20 x confirm_overall + 0.10 x buyback_score)).</t>
         </is>
       </c>
     </row>
@@ -712,7 +712,7 @@
       </c>
       <c r="D20" s="8" t="inlineStr">
         <is>
-          <t>3,746</t>
+          <t>3,747</t>
         </is>
       </c>
       <c r="E20" s="8" t="inlineStr">
@@ -1392,7 +1392,7 @@
         </is>
       </c>
       <c r="K10" s="22" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="L10" s="22" t="n">
         <v>3</v>
@@ -1872,7 +1872,7 @@
         </is>
       </c>
       <c r="K18" s="22" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="L18" s="22" t="n">
         <v>3</v>
@@ -2112,7 +2112,7 @@
         </is>
       </c>
       <c r="K22" s="22" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="L22" s="22" t="n">
         <v>3</v>
@@ -2172,7 +2172,7 @@
         </is>
       </c>
       <c r="K23" s="22" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="L23" s="22" t="n">
         <v>3</v>
@@ -2712,7 +2712,7 @@
         </is>
       </c>
       <c r="K32" s="22" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="L32" s="22" t="n">
         <v>3</v>
@@ -2772,7 +2772,7 @@
         </is>
       </c>
       <c r="K33" s="22" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="L33" s="22" t="n">
         <v>3</v>
@@ -3552,7 +3552,7 @@
         </is>
       </c>
       <c r="K46" s="22" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="L46" s="22" t="n">
         <v>6</v>
@@ -3612,7 +3612,7 @@
         </is>
       </c>
       <c r="K47" s="22" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="L47" s="22" t="n">
         <v>3</v>
@@ -3788,7 +3788,7 @@
         </is>
       </c>
       <c r="K50" s="22" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="L50" s="22" t="n">
         <v>3</v>
@@ -4388,7 +4388,7 @@
         </is>
       </c>
       <c r="K60" s="22" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="L60" s="22" t="n">
         <v>3</v>
@@ -4508,7 +4508,7 @@
         </is>
       </c>
       <c r="K62" s="22" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="L62" s="22" t="n">
         <v>3</v>
@@ -4688,7 +4688,7 @@
         </is>
       </c>
       <c r="K65" s="22" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="L65" s="22" t="n">
         <v>3</v>
@@ -4928,7 +4928,7 @@
         </is>
       </c>
       <c r="K69" s="22" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="L69" s="22" t="n">
         <v>3</v>
@@ -5048,7 +5048,7 @@
         </is>
       </c>
       <c r="K71" s="22" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="L71" s="22" t="n">
         <v>3</v>
@@ -5648,7 +5648,7 @@
         </is>
       </c>
       <c r="K81" s="22" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="L81" s="22" t="n">
         <v>5</v>
@@ -6428,7 +6428,7 @@
         </is>
       </c>
       <c r="K94" s="22" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L94" s="22" t="n">
         <v>3</v>
@@ -8528,7 +8528,7 @@
         </is>
       </c>
       <c r="K129" s="22" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="L129" s="22" t="n">
         <v>3</v>
@@ -10560,7 +10560,7 @@
         </is>
       </c>
       <c r="K163" s="22" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="L163" s="22" t="n">
         <v>4</v>
@@ -11160,7 +11160,7 @@
         </is>
       </c>
       <c r="K173" s="22" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="L173" s="22" t="n">
         <v>4</v>
@@ -11280,7 +11280,7 @@
         </is>
       </c>
       <c r="K175" s="22" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="L175" s="22" t="n">
         <v>3</v>
@@ -11696,7 +11696,7 @@
         </is>
       </c>
       <c r="K182" s="22" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L182" s="22" t="n">
         <v>5</v>
@@ -12292,7 +12292,7 @@
         </is>
       </c>
       <c r="K192" s="22" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="L192" s="22" t="n">
         <v>3</v>
@@ -15783,7 +15783,7 @@
         </is>
       </c>
       <c r="K38" s="22" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L38" s="22" t="n">
         <v>3</v>
@@ -16743,7 +16743,7 @@
         </is>
       </c>
       <c r="K54" s="22" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="L54" s="22" t="n">
         <v>3</v>
@@ -18063,7 +18063,7 @@
         </is>
       </c>
       <c r="K76" s="22" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="L76" s="22" t="n">
         <v>3</v>
@@ -21239,7 +21239,7 @@
         </is>
       </c>
       <c r="K129" s="22" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="L129" s="22" t="n">
         <v>5</v>
@@ -26158,7 +26158,7 @@
         </is>
       </c>
       <c r="K11" s="22" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="L11" s="22" t="n">
         <v>0</v>
@@ -26634,7 +26634,7 @@
         </is>
       </c>
       <c r="K19" s="22" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="L19" s="22" t="n">
         <v>2</v>
@@ -27710,7 +27710,7 @@
         </is>
       </c>
       <c r="K37" s="22" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="L37" s="22" t="n">
         <v>2</v>
@@ -27942,7 +27942,7 @@
         </is>
       </c>
       <c r="K41" s="22" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="L41" s="22" t="n">
         <v>2</v>
@@ -28302,7 +28302,7 @@
         </is>
       </c>
       <c r="K47" s="22" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="L47" s="22" t="n">
         <v>2</v>
@@ -28422,7 +28422,7 @@
         </is>
       </c>
       <c r="K49" s="22" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="L49" s="22" t="n">
         <v>2</v>
@@ -28658,7 +28658,7 @@
         </is>
       </c>
       <c r="K53" s="22" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="L53" s="22" t="n">
         <v>2</v>
@@ -29434,7 +29434,7 @@
         </is>
       </c>
       <c r="K66" s="22" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="L66" s="22" t="n">
         <v>2</v>
@@ -29554,7 +29554,7 @@
         </is>
       </c>
       <c r="K68" s="22" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="L68" s="22" t="n">
         <v>2</v>
@@ -29614,7 +29614,7 @@
         </is>
       </c>
       <c r="K69" s="22" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="L69" s="22" t="n">
         <v>2</v>
@@ -31166,7 +31166,7 @@
         </is>
       </c>
       <c r="K95" s="22" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="L95" s="22" t="n">
         <v>2</v>
@@ -31814,7 +31814,7 @@
         </is>
       </c>
       <c r="K106" s="22" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="L106" s="22" t="n">
         <v>2</v>
@@ -32350,7 +32350,7 @@
         </is>
       </c>
       <c r="K115" s="22" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="L115" s="22" t="n">
         <v>2</v>
@@ -32410,7 +32410,7 @@
         </is>
       </c>
       <c r="K116" s="22" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="L116" s="22" t="n">
         <v>2</v>
@@ -32586,7 +32586,7 @@
         </is>
       </c>
       <c r="K119" s="22" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="L119" s="22" t="n">
         <v>1</v>
@@ -32946,7 +32946,7 @@
         </is>
       </c>
       <c r="K125" s="22" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="L125" s="22" t="n">
         <v>0</v>
@@ -33366,7 +33366,7 @@
         </is>
       </c>
       <c r="K132" s="22" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="L132" s="22" t="n">
         <v>2</v>
@@ -34202,7 +34202,7 @@
         </is>
       </c>
       <c r="K146" s="22" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="L146" s="22" t="n">
         <v>2</v>
@@ -35282,7 +35282,7 @@
         </is>
       </c>
       <c r="K164" s="22" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L164" s="22" t="n">
         <v>2</v>
@@ -35878,7 +35878,7 @@
         </is>
       </c>
       <c r="K174" s="22" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="L174" s="22" t="n">
         <v>2</v>
@@ -36474,7 +36474,7 @@
         </is>
       </c>
       <c r="K184" s="22" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L184" s="22" t="n">
         <v>2</v>
@@ -37614,7 +37614,7 @@
         </is>
       </c>
       <c r="K203" s="22" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L203" s="22" t="n">
         <v>1</v>
@@ -38034,7 +38034,7 @@
         </is>
       </c>
       <c r="K210" s="22" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="L210" s="22" t="n">
         <v>2</v>
@@ -38154,7 +38154,7 @@
         </is>
       </c>
       <c r="K212" s="22" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="L212" s="22" t="n">
         <v>1</v>
@@ -38334,7 +38334,7 @@
         </is>
       </c>
       <c r="K215" s="22" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="L215" s="22" t="n">
         <v>1</v>
@@ -39114,7 +39114,7 @@
         </is>
       </c>
       <c r="K228" s="22" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="L228" s="22" t="n">
         <v>0</v>
@@ -39830,7 +39830,7 @@
         </is>
       </c>
       <c r="K240" s="22" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="L240" s="22" t="n">
         <v>1</v>
@@ -40310,7 +40310,7 @@
         </is>
       </c>
       <c r="K248" s="22" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="L248" s="22" t="n">
         <v>2</v>
@@ -42406,7 +42406,7 @@
         </is>
       </c>
       <c r="K283" s="22" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="L283" s="22" t="n">
         <v>2</v>
@@ -43062,7 +43062,7 @@
         </is>
       </c>
       <c r="K294" s="22" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="L294" s="22" t="n">
         <v>0</v>
@@ -43182,7 +43182,7 @@
         </is>
       </c>
       <c r="K296" s="22" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L296" s="22" t="n">
         <v>0</v>
@@ -43418,14 +43418,14 @@
         </is>
       </c>
       <c r="K300" s="22" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L300" s="22" t="n">
         <v>0</v>
       </c>
       <c r="M300" s="21" t="inlineStr">
         <is>
-          <t>NetCashReturner, StrongCoverage, LynchPEGY</t>
+          <t>NetCashReturner, StrongCoverage, LynchPEGY, Greenblatt-MagicFormula</t>
         </is>
       </c>
       <c r="N300" s="24" t="n">
@@ -43598,7 +43598,7 @@
         </is>
       </c>
       <c r="K303" s="22" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="L303" s="22" t="n">
         <v>1</v>
@@ -44078,7 +44078,7 @@
         </is>
       </c>
       <c r="K311" s="22" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="L311" s="22" t="n">
         <v>2</v>
@@ -45454,7 +45454,7 @@
         </is>
       </c>
       <c r="K334" s="22" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="L334" s="22" t="n">
         <v>1</v>
@@ -46114,7 +46114,7 @@
         </is>
       </c>
       <c r="K345" s="22" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="L345" s="22" t="n">
         <v>1</v>
@@ -46946,7 +46946,7 @@
         </is>
       </c>
       <c r="K359" s="22" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="L359" s="22" t="n">
         <v>1</v>
@@ -47426,7 +47426,7 @@
         </is>
       </c>
       <c r="K367" s="22" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L367" s="22" t="n">
         <v>0</v>
@@ -49106,7 +49106,7 @@
         </is>
       </c>
       <c r="K395" s="22" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="L395" s="22" t="n">
         <v>1</v>
@@ -50546,7 +50546,7 @@
         </is>
       </c>
       <c r="K419" s="22" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L419" s="22" t="n">
         <v>0</v>
@@ -50722,7 +50722,7 @@
         </is>
       </c>
       <c r="K422" s="22" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L422" s="22" t="n">
         <v>2</v>
@@ -51442,7 +51442,7 @@
         </is>
       </c>
       <c r="K434" s="22" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="L434" s="22" t="n">
         <v>1</v>
@@ -51562,7 +51562,7 @@
         </is>
       </c>
       <c r="K436" s="22" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="L436" s="22" t="n">
         <v>1</v>
@@ -52762,7 +52762,7 @@
         </is>
       </c>
       <c r="K456" s="22" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="L456" s="22" t="n">
         <v>2</v>
@@ -52882,7 +52882,7 @@
         </is>
       </c>
       <c r="K458" s="22" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="L458" s="22" t="n">
         <v>2</v>
@@ -52942,14 +52942,14 @@
         </is>
       </c>
       <c r="K459" s="22" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L459" s="22" t="n">
         <v>2</v>
       </c>
       <c r="M459" s="21" t="inlineStr">
         <is>
-          <t>MidCapGARP, Bottleneck-Chokepoint, Flyover-QuietQuality</t>
+          <t>MidCapGARP, Bottleneck-Chokepoint, Flyover-QuietQuality, Greenblatt-Ma</t>
         </is>
       </c>
       <c r="N459" s="24" t="n">
@@ -54922,7 +54922,7 @@
         </is>
       </c>
       <c r="K492" s="22" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L492" s="22" t="n">
         <v>1</v>

</xml_diff>

<commit_message>
Rebuild all books with the two new XR forensic archetypes
Regenerated the render-managed workbooks so arch_xr_oneoff_loss_mask (83) and
arch_xr_monetization_trifecta (9) surface across the archetype, country,
segment, and top-N books.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Pk8K7QpC1m36MYjRwkTznS
</commit_message>
<xml_diff>
--- a/nms_multibagger_candidates_midcap_plus.xlsx
+++ b/nms_multibagger_candidates_midcap_plus.xlsx
@@ -658,7 +658,7 @@
     <row r="9" ht="22" customHeight="1">
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>This shortlist filters the 4,208 multibagger candidates in the NMS sub-universe (mcap &lt; ~$2B, RED-verdicted names excluded). Each name is assigned a conviction tier based on its archetype-count, inflection-cluster density and asymmetry score. STRICT (217) = 5+ archetypes firing AND 3+ inflection signals AND asymmetry &gt;= 0.40. STRONG (216) = 3+ archetypes AND 3+ inflection signals AND asymmetry &gt;= 0.35. CANDIDATE (3775) = the broader funnel - 3+ archetypes or 4+ inflection signals at asymmetry &gt;= 0.35. (Multi-archetype gates are calibrated to the current 69-archetype taxonomy.) Within each tier, names are ranked by confirmed entry-today asymmetry (asymmetry_score x qual_multiplier x post-rally factor x confirmation multiplier (1 + 0.20 x confirm_overall + 0.10 x buyback_score)).</t>
+          <t>This shortlist filters the 4,211 multibagger candidates in the NMS sub-universe (mcap &lt; ~$2B, RED-verdicted names excluded). Each name is assigned a conviction tier based on its archetype-count, inflection-cluster density and asymmetry score. STRICT (217) = 5+ archetypes firing AND 3+ inflection signals AND asymmetry &gt;= 0.40. STRONG (216) = 3+ archetypes AND 3+ inflection signals AND asymmetry &gt;= 0.35. CANDIDATE (3778) = the broader funnel - 3+ archetypes or 4+ inflection signals at asymmetry &gt;= 0.35. (Multi-archetype gates are calibrated to the current 69-archetype taxonomy.) Within each tier, names are ranked by confirmed entry-today asymmetry (asymmetry_score x qual_multiplier x post-rally factor x confirmation multiplier (1 + 0.20 x confirm_overall + 0.10 x buyback_score)).</t>
         </is>
       </c>
     </row>
@@ -712,7 +712,7 @@
       </c>
       <c r="D20" s="8" t="inlineStr">
         <is>
-          <t>3,775</t>
+          <t>3,778</t>
         </is>
       </c>
       <c r="E20" s="8" t="inlineStr">

</xml_diff>

<commit_message>
Rebuild all books with deep-trough double_trough (298 firers)
Regenerated the render-managed workbooks so arch_xr_double_trough's newly
admitted deep (negative-EBITDA, fortress-balance-sheet) troughs surface.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Pk8K7QpC1m36MYjRwkTznS
</commit_message>
<xml_diff>
--- a/nms_multibagger_candidates_midcap_plus.xlsx
+++ b/nms_multibagger_candidates_midcap_plus.xlsx
@@ -658,7 +658,7 @@
     <row r="9" ht="22" customHeight="1">
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>This shortlist filters the 4,211 multibagger candidates in the NMS sub-universe (mcap &lt; ~$2B, RED-verdicted names excluded). Each name is assigned a conviction tier based on its archetype-count, inflection-cluster density and asymmetry score. STRICT (217) = 5+ archetypes firing AND 3+ inflection signals AND asymmetry &gt;= 0.40. STRONG (216) = 3+ archetypes AND 3+ inflection signals AND asymmetry &gt;= 0.35. CANDIDATE (3778) = the broader funnel - 3+ archetypes or 4+ inflection signals at asymmetry &gt;= 0.35. (Multi-archetype gates are calibrated to the current 69-archetype taxonomy.) Within each tier, names are ranked by confirmed entry-today asymmetry (asymmetry_score x qual_multiplier x post-rally factor x confirmation multiplier (1 + 0.20 x confirm_overall + 0.10 x buyback_score)).</t>
+          <t>This shortlist filters the 4,212 multibagger candidates in the NMS sub-universe (mcap &lt; ~$2B, RED-verdicted names excluded). Each name is assigned a conviction tier based on its archetype-count, inflection-cluster density and asymmetry score. STRICT (217) = 5+ archetypes firing AND 3+ inflection signals AND asymmetry &gt;= 0.40. STRONG (216) = 3+ archetypes AND 3+ inflection signals AND asymmetry &gt;= 0.35. CANDIDATE (3779) = the broader funnel - 3+ archetypes or 4+ inflection signals at asymmetry &gt;= 0.35. (Multi-archetype gates are calibrated to the current 69-archetype taxonomy.) Within each tier, names are ranked by confirmed entry-today asymmetry (asymmetry_score x qual_multiplier x post-rally factor x confirmation multiplier (1 + 0.20 x confirm_overall + 0.10 x buyback_score)).</t>
         </is>
       </c>
     </row>
@@ -712,7 +712,7 @@
       </c>
       <c r="D20" s="8" t="inlineStr">
         <is>
-          <t>3,778</t>
+          <t>3,779</t>
         </is>
       </c>
       <c r="E20" s="8" t="inlineStr">

</xml_diff>